<commit_message>
Add accessibility test & cover max-10 cart limit
</commit_message>
<xml_diff>
--- a/docs/Test_Cases_UI.xlsx
+++ b/docs/Test_Cases_UI.xlsx
@@ -10,7 +10,7 @@
     <sheet name="UI Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UI Test Cases'!$A$1:$K$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UI Test Cases'!$A$1:$K$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1230,8 +1230,67 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-17</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Кошик</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Кількість обмежена максимумом 10, навіть якщо stock більший</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Створено нове середовище; у кошику p05 × 9</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>p05 «Термопляшка «Щодня»» (stock 20); кількості 9 → 10 → 11</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити кошик
+2. Натиснути «+» біля p05
+3. Спробувати натиснути «+» ще раз</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Кількість стає 10; кнопка «+» неактивна, 11 встановити неможливо</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>🆕 Додано після повторної звірки з ТЗ. ТЗ: «Кількість 1–10, не більше stock». TC-UI-5 упирається в stock p01 (8) раніше, ніж у 10, тому межу 10 перевіряємо на p05 (stock 20).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K13"/>
+  <autoFilter ref="A1:K14"/>
   <dataValidations count="2">
     <dataValidation sqref="I2:I213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Оберіть значення зі списку" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>

</xml_diff>

<commit_message>
Add network error tests (TC-UI-18…22) and BUG-8 duplicate cart line
</commit_message>
<xml_diff>
--- a/docs/Test_Cases_UI.xlsx
+++ b/docs/Test_Cases_UI.xlsx
@@ -10,7 +10,7 @@
     <sheet name="UI Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UI Test Cases'!$A$1:$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UI Test Cases'!$A$1:$K$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1289,8 +1289,67 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-23</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Кошик</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Повторне додавання того самого товару не створює другу позицію (p07)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Створено нове середовище; кошик порожній</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>p07 «Таймер «Фокус»» (750 грн, stock 3, 2-га сторінка каталогу)</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>1. Перейти на 2-гу сторінку каталогу
+2. Двічі натиснути «До кошика» на p07
+3. Відкрити кошик</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>У кошику одна позиція p07 з кількістю 2</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>У кошику дві окремі позиції p07 по 1 шт. Замовлення при цьому оформлюється коректно (сайт об'єднує позиції перед відправкою). Дефект BUG-8</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>🆕 Додано для BUG-8. ТЗ: «Одна позиція на product_id». TC-UI-5 перевіряє правило лише на p01, дефект проявляється на p07.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K14"/>
+  <autoFilter ref="A1:K15"/>
   <dataValidations count="2">
     <dataValidation sqref="I2:I213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Оберіть значення зі списку" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>

</xml_diff>

<commit_message>
Merge accessibility and network test cases into Test_Cases_UI.xlsx
</commit_message>
<xml_diff>
--- a/docs/Test_Cases_UI.xlsx
+++ b/docs/Test_Cases_UI.xlsx
@@ -10,7 +10,7 @@
     <sheet name="UI Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UI Test Cases'!$A$1:$K$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UI Test Cases'!$A$1:$K$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1233,123 +1233,660 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>TC-UI-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Доступність</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Немає критичних і серйозних порушень WCAG 2.1 AA (axe-core)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Створено нове середовище; у кошику p01 × 1</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Правила axe-core з тегами wcag2a, wcag2aa, wcag21a, wcag21aa; блокуючі рівні — critical і serious</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити каталог і запустити аудит усієї сторінки
+2. Відкрити картку товару p02 і перевірити діалог
+3. Відкрити кошик і перевірити діалог із формою оформлення
+4. Натиснути «Почати заново» і перевірити діалог підтвердження</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>У кожному стані немає порушень рівня critical або serious</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Каталог: label-content-name-mismatch [serious] × 2 — кнопки «← Назад» / «Далі →» мають aria-label «Попередня / Наступна сторінка», що не містить видимого тексту. Дефект BUG-7. Решта станів відповідає очікуваному</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>🆕 ТЗ: «завдання з зірочкою — доступність». WCAG 2.1 AA — загальноприйнятий стандарт; axe-core перевіряє ту частину правил, яку можна автоматизувати.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Доступність</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Поля форм мають підписи, кнопки-іконки мають доступні назви</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Створено нове середовище; у кошику p01 × 1</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Поля: #search, #sort, #min-price, #max-price, #coupon, #delivery, #customer-name, #email, #address, #payment; кнопки «♡», «−», «+», «×»</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>1. Перевірити, що кожне поле фільтрів і оформлення має &lt;label&gt; або aria-label
+2. Перевірити aria-label кнопки «♡» на p01 і її стан aria-pressed до й після натискання
+3. Відкрити кошик і перевірити aria-label кнопок «−», «+» і «×»
+4. Перевірити role="alert" у помилки оформлення і aria-live у повідомлень</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Усі поля мають підпис; кнопки-іконки мають назву; aria-pressed змінюється false → true; помилки й повідомлення озвучуються</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>🆕 ТЗ: «підписи полів». Підпис рахується і через &lt;label for&gt;, і через &lt;label&gt;, що обгортає поле (так зроблено в полі пошуку).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Доступність</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Оформлення замовлення лише з клавіатури</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Створено нове середовище; кошик порожній</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>p01 × 1; ім'я «Олександр Тестовий», email test@example.test, адреса «Київ, вул. Тестова, 12»; «Успішна оплата»</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>1. Перевести фокус на «До кошика» в p01 і натиснути Enter
+2. Перевести фокус на «Кошик» і натиснути Enter
+3. Ввести ім'я, натиснути Tab; ввести email, натиснути Tab; ввести адресу, натиснути Tab
+4. Перевести фокус на «Оформити замовлення» і натиснути Enter</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Товар додано (лічильник 1); кошик відкрився; Tab переходить ім'я → email → адреса → оплата; замовлення створено (201, у списку одне замовлення)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>🆕 ТЗ: «клавіатурна навігація». Клавіші натискаються через Chrome DevTools Protocol (cypress-real-events), як справжня клавіатура.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Доступність</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Діалоги закриваються Esc і повертають фокус</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Створено нове середовище; у кошику p01 × 1</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Діалоги: кошик (#bag-dialog), картка товару p02 (#product-dialog)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>1. Перевести фокус на «Кошик», натиснути Enter
+2. Натиснути Esc
+3. Перевести фокус на назву товару p02, натиснути Enter
+4. Натиснути Esc</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Діалог відкривається, фокус усередині діалогу; Esc закриває його; фокус повертається на кнопку, яка відкрила діалог</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>🆕 ТЗ: «клавіатурна навігація». Без повернення фокуса користувач клавіатури після закриття діалогу опиняється на початку сторінки.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>TC-UI-17</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Кошик</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Кількість обмежена максимумом 10, навіть якщо stock більший</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Створено нове середовище; у кошику p05 × 9</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>p05 «Термопляшка «Щодня»» (stock 20); кількості 9 → 10 → 11</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>1. Відкрити кошик
 2. Натиснути «+» біля p05
 3. Спробувати натиснути «+» ще раз</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Кількість стає 10; кнопка «+» неактивна, 11 встановити неможливо</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Відповідає очікуваному результату</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>🆕 Додано після повторної звірки з ТЗ. ТЗ: «Кількість 1–10, не більше stock». TC-UI-5 упирається в stock p01 (8) раніше, ніж у 10, тому межу 10 перевіряємо на p05 (stock 20).</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Мережеві помилки</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Каталог показує стани завантаження й помилки та відновлюється</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Сайт відкрито в новому середовищі</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Категорія «Аудіо», потім «Робочий простір»; затримка відповіді 1,5 с; обрив мережі; відповідь 500</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>1. Уповільнити відповідь каталогу й обрати «Аудіо»
+2. Дочекатися відповіді
+3. Імітувати обрив мережі й обрати «Аудіо»; відновити мережу
+4. Обрати «Робочий простір»
+5. Повторити кроки 3–4 з відповіддю сервера 500</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>1: показано «Завантажуємо товари…», aria-busy=true. 2: 3 товари, aria-busy=false. 3: повідомлення «Немає зв’язку із сервером…», безкінечного завантаження немає. 4: товари знову завантажились. 5: повідомлення з кодом 500, далі відновлення</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>🆕 ТЗ: «стани завантаження/помилки». Обрив мережі імітується офлайн-режимом браузера (DevTools Protocol); помилка сервера — відповіддю 500 через cy.intercept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Мережеві помилки</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Оформлення замовлення переживає збій мережі</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Нове середовище; p01 у кошику</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>p01 × 1; ім'я «Олександр Тестовий», email test@example.test, адреса «Київ, вул. Тестова, 12»; «Успішна оплата»; обрив мережі або відповідь 500</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити кошик і заповнити контакти
+2. Імітувати збій і натиснути «Оформити замовлення»
+3. Відновити мережу; перевірити кошик, форму й список замовлень
+4. Ще раз натиснути «Оформити замовлення»</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2: показано помилку (role=alert). 3: кошик і введені дані збереглися, кнопка активна, замовлення не створено. 4: створено рівно одне замовлення</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>🆕 Найкритичніший крок: збій не повинен ні загубити кошик, ні створити «фантомне» замовлення. Перевіряються обидва види збою.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Мережеві помилки</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Суми не показуються, а оформлення заблоковане, поки розрахунок падає</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Нове середовище; p01 у кошику</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>p01 × 1 (2 400 грн); відповідь 500 на POST /api/quote; потім експрес-доставка</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>1. Імітувати 500 на розрахунок і відкрити кошик
+2. Перевірити блок сум і кнопку оформлення
+3. Обрати експрес-доставку (мережа в нормі)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>1–2: показано помилку з кодом 500; суми («Разом») не показані; кнопка «Оформити замовлення» неактивна. 3: суми з'явились (разом 2 550 грн), кнопка активна</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>🆕 Користувач не повинен оформлювати замовлення з невідомою або застарілою сумою.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Мережеві помилки</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Невдале збереження обраного не показується як збережене</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Нове середовище</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Товар p01; обрив мережі під час збереження</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>1. Імітувати обрив мережі й натиснути «♡» на p01
+2. Відновити мережу; перевірити кнопку й обране на сервері</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Показано повідомлення «Немає зв’язку…»; кнопка лишилась aria-pressed=false; на сервері обране порожнє</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>🆕 ТЗ: обране зберігається на сервері, тож інтерфейс не має показувати збереження, якого не було.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Стани UI</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Стани порожніх даних</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Нове середовище</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Пошуковий запит «немає-такого-товару»; нове середовище без замовлень і обраного</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>1. Ввести в пошук «немає-такого-товару»
+2. Відкрити «Мої замовлення»
+3. Відкрити «Обране»</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>1: «Тут поки порожньо». 2: «Замовлень не знайдено». 3: показано порожній стан, а не порожню область</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>🆕 ТЗ: «стани … порожніх даних».</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>TC-UI-23</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Кошик</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Повторне додавання того самого товару не створює другу позицію (p07)</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Створено нове середовище; кошик порожній</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>p07 «Таймер «Фокус»» (750 грн, stock 3, 2-га сторінка каталогу)</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>1. Перейти на 2-гу сторінку каталогу
 2. Двічі натиснути «До кошика» на p07
 3. Відкрити кошик</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>У кошику одна позиція p07 з кількістю 2</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>У кошику дві окремі позиції p07 по 1 шт. Замовлення при цьому оформлюється коректно (сайт об'єднує позиції перед відправкою). Дефект BUG-8</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>🆕 Додано для BUG-8. ТЗ: «Одна позиція на product_id». TC-UI-5 перевіряє правило лише на p01, дефект проявляється на p07.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K15"/>
+  <autoFilter ref="A1:K24"/>
   <dataValidations count="2">
     <dataValidation sqref="I2:I213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Оберіть значення зі списку" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>

</xml_diff>

<commit_message>
Add mobile test + fix TC-UI-3 race and TC-UI-15 flakiness, bound 429 retries, remove dead code
</commit_message>
<xml_diff>
--- a/docs/Test_Cases_UI.xlsx
+++ b/docs/Test_Cases_UI.xlsx
@@ -10,7 +10,7 @@
     <sheet name="UI Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UI Test Cases'!$A$1:$K$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'UI Test Cases'!$A$1:$K$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1885,8 +1885,246 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Мобільний режим</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Немає горизонтального скролу сторінки на ключових екранах</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Нове середовище з одним замовленням; у кошику p01 × 1</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Ширина екрана 360×780 (мінімум за ТЗ) і 768×1024 (планшет)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити каталог
+2. Відкрити картку товару p02
+3. Відкрити кошик
+4. Відкрити «Мої замовлення»</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>На кожному екрані ширина сторінки не перевищує ширину вікна — сторінка не прокручується вбік</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>🆕 Завдання з зірочкою — мобільний режим. ТЗ: «Адаптивність від 360px». Перевірку підтверджено контрольним прогоном: штучно широкий елемент тест ловить.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Мобільний режим</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Навігація в шапці поміщається на екрані й працює</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Сайт відкрито; ширина 360×780</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Посилання «Обране», «Мої замовлення», кнопка «Кошик»</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>1. Перевірити, що «Обране», «Мої замовлення» і «Кошик» видимі й не обрізані краєм екрана
+2. Перейти в «Мої замовлення»</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Усі елементи шапки видимі в межах екрана; відкривається розділ «Мої замовлення»</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>🆕 Завдання з зірочкою — мобільний режим. Без доступної навігації на телефоні неможливо дістатися кошика й замовлень.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Мобільний режим</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Діалоги вміщаються в екран; широкий вміст прокручується всередині діалогу</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Ширина 360×780; у кошику p01 × 1; у порівнянні p01, p02</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Діалоги кошика й порівняння</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити кошик; перевірити межі діалогу і кнопки «×»
+2. Прокрутити до «Оформити замовлення»
+3. Закрити кошик і відкрити порівняння
+4. Перевірити таблицю порівняння і сторінку</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Діалоги й кнопка закриття в межах екрана; кнопка оформлення досяжна прокруткою; таблиця порівняння прокручується у власному контейнері, сторінка вбік не прокручується</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>🆕 Завдання з зірочкою — мобільний режим. Таблиця порівняння ширша за 360px — це очікувано; важливо, що вона не розтягує сторінку.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TC-UI-27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Мобільний режим</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Оформлення замовлення на екрані 360px</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Нове середовище; кошик порожній; ширина 360×780</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>p01 × 1 (2 400 грн); промокод WELCOME10; ім'я «Олександр Тестовий», email test@example.test, адреса «Київ, вул. Тестова, 12»; «Успішна оплата»</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>1. Додати p01 до кошика
+2. Відкрити кошик і застосувати WELCOME10
+3. Заповнити контакти
+4. Прокрутити до кнопки й оформити замовлення</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Лічильник кошика 1; разом 2 160 грн; замовлення створено (201), показано повідомлення про успіх, у списку одне замовлення</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Відповідає очікуваному результату</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>🆕 Завдання з зірочкою — мобільний режим. Основний сценарій покупки (як TC-UI-1) на мінімальній ширині з ТЗ.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K24"/>
+  <autoFilter ref="A1:K28"/>
   <dataValidations count="2">
     <dataValidation sqref="I2:I213" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Оберіть значення зі списку" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>

</xml_diff>